<commit_message>
Refresh aggregate/*.xlsx after pulling latest flan-t5-base results
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YaN74QjRwggrFfWuN5JEVJ
</commit_message>
<xml_diff>
--- a/analysis/aggregate/ac-PRF.xlsx
+++ b/analysis/aggregate/ac-PRF.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>t5-base</t>
+          <t>flan-t5-base</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -518,22 +518,22 @@
         <v>5</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7979117605724549</v>
+        <v>0.7628361810666193</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02630474341726022</v>
+        <v>0.01158194176832889</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7929411764705883</v>
+        <v>0.7564705882352941</v>
       </c>
       <c r="K2" t="n">
-        <v>0.02054617552538</v>
+        <v>0.008921029934178263</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7953442886268538</v>
+        <v>0.7596117747476989</v>
       </c>
       <c r="M2" t="n">
-        <v>0.02196473464022954</v>
+        <v>0.008927422050968992</v>
       </c>
     </row>
     <row r="3">
@@ -544,7 +544,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>t5-base</t>
+          <t>flan-t5-base</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -571,22 +571,22 @@
         <v>5</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7979117605724549</v>
+        <v>0.7019070427318238</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02630474341726022</v>
+        <v>0.0129895994446469</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7929411764705883</v>
+        <v>0.7035294117647058</v>
       </c>
       <c r="K3" t="n">
-        <v>0.02054617552538</v>
+        <v>0.0121979066784281</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7953442886268538</v>
+        <v>0.7027086223504331</v>
       </c>
       <c r="M3" t="n">
-        <v>0.02196473464022954</v>
+        <v>0.01230075357459118</v>
       </c>
     </row>
     <row r="4">
@@ -597,7 +597,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>t5-base</t>
+          <t>flan-t5-base</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -624,22 +624,22 @@
         <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7946384282584276</v>
+        <v>0.7645535610693981</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02215577199420941</v>
+        <v>0.01748613562702413</v>
       </c>
       <c r="J4" t="n">
-        <v>0.7905882352941177</v>
+        <v>0.76</v>
       </c>
       <c r="K4" t="n">
-        <v>0.01068582477916766</v>
+        <v>0.01464694070351614</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7925445230105735</v>
+        <v>0.762264620148735</v>
       </c>
       <c r="M4" t="n">
-        <v>0.01535006605215245</v>
+        <v>0.01595534167926884</v>
       </c>
     </row>
     <row r="5">
@@ -650,7 +650,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>t5-base</t>
+          <t>flan-t5-base</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -677,22 +677,22 @@
         <v>5</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7946384282584276</v>
+        <v>0.6978614358393845</v>
       </c>
       <c r="I5" t="n">
-        <v>0.02215577199420941</v>
+        <v>0.02486904288646526</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7905882352941177</v>
+        <v>0.7035294117647058</v>
       </c>
       <c r="K5" t="n">
-        <v>0.01068582477916766</v>
+        <v>0.02338189048747269</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7925445230105735</v>
+        <v>0.7006680369052052</v>
       </c>
       <c r="M5" t="n">
-        <v>0.01535006605215245</v>
+        <v>0.02384425735629462</v>
       </c>
     </row>
     <row r="6">
@@ -703,7 +703,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>t5-base</t>
+          <t>flan-t5-base</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -727,25 +727,25 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8186567456362652</v>
+        <v>0.7909247228180893</v>
       </c>
       <c r="I6" t="n">
-        <v>0.007220599924965905</v>
+        <v>0.01388019588585022</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8057142857142857</v>
+        <v>0.7691428571428572</v>
       </c>
       <c r="K6" t="n">
-        <v>0.008081220356417699</v>
+        <v>0.01315527363796723</v>
       </c>
       <c r="L6" t="n">
-        <v>0.812091021285785</v>
+        <v>0.7798398540520636</v>
       </c>
       <c r="M6" t="n">
-        <v>0.003552758547473675</v>
+        <v>0.01190036491214692</v>
       </c>
     </row>
     <row r="7">
@@ -756,7 +756,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>t5-base</t>
+          <t>flan-t5-base</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -783,22 +783,22 @@
         <v>5</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8162890328726485</v>
+        <v>0.7909247228180893</v>
       </c>
       <c r="I7" t="n">
-        <v>0.008193480097753366</v>
+        <v>0.01388019588585022</v>
       </c>
       <c r="J7" t="n">
-        <v>0.8068571428571427</v>
+        <v>0.7691428571428572</v>
       </c>
       <c r="K7" t="n">
-        <v>0.007450517034517296</v>
+        <v>0.01315527363796723</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8114961788519899</v>
+        <v>0.7798398540520636</v>
       </c>
       <c r="M7" t="n">
-        <v>0.003351978158894027</v>
+        <v>0.01190036491214692</v>
       </c>
     </row>
     <row r="8">
@@ -809,7 +809,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>t5-base</t>
+          <t>flan-t5-base</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -836,22 +836,22 @@
         <v>5</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8157392026578073</v>
+        <v>0.7499324435148262</v>
       </c>
       <c r="I8" t="n">
-        <v>0.01143414204462839</v>
+        <v>0.02668125337544833</v>
       </c>
       <c r="J8" t="n">
-        <v>0.7942857142857143</v>
+        <v>0.7588571428571429</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0193780856660722</v>
+        <v>0.01779704171702564</v>
       </c>
       <c r="L8" t="n">
-        <v>0.8047992775629075</v>
+        <v>0.7542292479962034</v>
       </c>
       <c r="M8" t="n">
-        <v>0.01364890851437444</v>
+        <v>0.01966583541848766</v>
       </c>
     </row>
     <row r="9">
@@ -862,48 +862,472 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>flan-t5-base</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>paraphrase</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.7499324435148262</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.02668125337544833</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.7588571428571429</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.01779704171702564</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.7542292479962034</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.01966583541848766</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>acos_drone_binary</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>t5-base</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>gen-scl-nat</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.7979117605724549</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.02630474341726022</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.7929411764705883</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.02054617552538</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.7953442886268538</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.02196473464022954</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>acos_drone_binary</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>t5-base</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>gen-scl-nat</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.7979117605724549</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.02630474341726022</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.7929411764705883</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.02054617552538</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.7953442886268538</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.02196473464022954</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>acos_drone_binary</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>t5-base</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>gen-scl-nat</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.7946384282584276</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.02215577199420941</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.7905882352941177</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.01068582477916766</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.7925445230105735</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.01535006605215245</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>acos_drone_binary</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>t5-base</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>gen-scl-nat</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.7946384282584276</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.02215577199420941</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.7905882352941177</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.01068582477916766</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.7925445230105735</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.01535006605215245</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>acos_drone_binary</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>t5-base</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>paraphrase</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>5</v>
-      </c>
-      <c r="H9" t="n">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.8186567456362652</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.007220599924965905</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.8057142857142857</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.008081220356417699</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.812091021285785</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.003552758547473675</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>acos_drone_binary</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>t5-base</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>paraphrase</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.8162890328726485</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.008193480097753366</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.8068571428571427</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.007450517034517296</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.8114961788519899</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.003351978158894027</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>acos_drone_binary</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>t5-base</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>paraphrase</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" t="n">
         <v>0.8157392026578073</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I16" t="n">
         <v>0.01143414204462839</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J16" t="n">
         <v>0.7942857142857143</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K16" t="n">
         <v>0.0193780856660722</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L16" t="n">
         <v>0.8047992775629075</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M16" t="n">
+        <v>0.01364890851437444</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>acos_drone_binary</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>t5-base</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>paraphrase</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.8157392026578073</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.01143414204462839</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.7942857142857143</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.0193780856660722</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.8047992775629075</v>
+      </c>
+      <c r="M17" t="n">
         <v>0.01364890851437444</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Test base_model as a Wilcoxon scenario axis; refresh analysis outputs
significance.py: base_model moves from GROUP_COLUMNS into
SCENARIO_COLUMNS (grouping is now dataset-only), with a new
--baseline_base_model flag (default t5-base), so flan-t5-base runs are
tested directly against the t5-base baseline like any other ablation,
instead of only ever being compared within their own base-model group.

recap/aggregate/statistics xlsx outputs regenerated against the full
80-run grid (2 base models x 2 templates x 2 contrastive x 2 CD x 5
seeds, all seg-off) now on disk after the dataset space-fix rerun and
the seed-reordering commit; the versions previously committed here
were stale (generated against the old seed-first layout and included
now-deleted segmentation runs).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YaN74QjRwggrFfWuN5JEVJ
</commit_message>
<xml_diff>
--- a/analysis/aggregate/ac-PRF.xlsx
+++ b/analysis/aggregate/ac-PRF.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -518,22 +518,22 @@
         <v>5</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7628361810666193</v>
+        <v>0.7759889143647976</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01158194176832889</v>
+        <v>0.03186679009088352</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7564705882352941</v>
+        <v>0.768235294117647</v>
       </c>
       <c r="K2" t="n">
-        <v>0.008921029934178263</v>
+        <v>0.02145245003389467</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7596117747476989</v>
+        <v>0.7720094910551094</v>
       </c>
       <c r="M2" t="n">
-        <v>0.008927422050968992</v>
+        <v>0.02560257284789822</v>
       </c>
     </row>
     <row r="3">
@@ -554,39 +554,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G3" t="n">
         <v>5</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7019070427318238</v>
+        <v>0.7702886756048087</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0129895994446469</v>
+        <v>0.01216676155822163</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7035294117647058</v>
+        <v>0.7647058823529411</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0121979066784281</v>
+        <v>0.01176470588235294</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7027086223504331</v>
+        <v>0.7674157623767675</v>
       </c>
       <c r="M3" t="n">
-        <v>0.01230075357459118</v>
+        <v>0.008565928406441768</v>
       </c>
     </row>
     <row r="4">
@@ -612,7 +612,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -624,22 +624,22 @@
         <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7645535610693981</v>
+        <v>0.7699335642954763</v>
       </c>
       <c r="I4" t="n">
-        <v>0.01748613562702413</v>
+        <v>0.02499191533635829</v>
       </c>
       <c r="J4" t="n">
-        <v>0.76</v>
+        <v>0.7623529411764707</v>
       </c>
       <c r="K4" t="n">
-        <v>0.01464694070351614</v>
+        <v>0.01642851769855169</v>
       </c>
       <c r="L4" t="n">
-        <v>0.762264620148735</v>
+        <v>0.7660446755512715</v>
       </c>
       <c r="M4" t="n">
-        <v>0.01595534167926884</v>
+        <v>0.01916198333272108</v>
       </c>
     </row>
     <row r="5">
@@ -670,29 +670,29 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G5" t="n">
         <v>5</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6978614358393845</v>
+        <v>0.7633106638694743</v>
       </c>
       <c r="I5" t="n">
-        <v>0.02486904288646526</v>
+        <v>0.01499691063642221</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7035294117647058</v>
+        <v>0.7623529411764706</v>
       </c>
       <c r="K5" t="n">
-        <v>0.02338189048747269</v>
+        <v>0.01354219345084862</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7006680369052052</v>
+        <v>0.7628121577403618</v>
       </c>
       <c r="M5" t="n">
-        <v>0.02384425735629462</v>
+        <v>0.01362949287380281</v>
       </c>
     </row>
     <row r="6">
@@ -730,22 +730,22 @@
         <v>5</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7909247228180893</v>
+        <v>0.7819833100010335</v>
       </c>
       <c r="I6" t="n">
-        <v>0.01388019588585022</v>
+        <v>0.01260262927311689</v>
       </c>
       <c r="J6" t="n">
-        <v>0.7691428571428572</v>
+        <v>0.7668571428571429</v>
       </c>
       <c r="K6" t="n">
-        <v>0.01315527363796723</v>
+        <v>0.0233517905619458</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7798398540520636</v>
+        <v>0.7742762991174907</v>
       </c>
       <c r="M6" t="n">
-        <v>0.01190036491214692</v>
+        <v>0.01710147790392485</v>
       </c>
     </row>
     <row r="7">
@@ -771,34 +771,34 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>5</v>
       </c>
       <c r="H7" t="n">
-        <v>0.7909247228180893</v>
+        <v>0.7731589839588976</v>
       </c>
       <c r="I7" t="n">
-        <v>0.01388019588585022</v>
+        <v>0.01314853035365245</v>
       </c>
       <c r="J7" t="n">
-        <v>0.7691428571428572</v>
+        <v>0.752</v>
       </c>
       <c r="K7" t="n">
-        <v>0.01315527363796723</v>
+        <v>0.01695131082764724</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7798398540520636</v>
+        <v>0.7624237094398205</v>
       </c>
       <c r="M7" t="n">
-        <v>0.01190036491214692</v>
+        <v>0.01495968233120615</v>
       </c>
     </row>
     <row r="8">
@@ -819,12 +819,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -836,22 +836,22 @@
         <v>5</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7499324435148262</v>
+        <v>0.7835981297285872</v>
       </c>
       <c r="I8" t="n">
-        <v>0.02668125337544833</v>
+        <v>0.00657014457145408</v>
       </c>
       <c r="J8" t="n">
-        <v>0.7588571428571429</v>
+        <v>0.7657142857142857</v>
       </c>
       <c r="K8" t="n">
-        <v>0.01779704171702564</v>
+        <v>0.01277753129999883</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7542292479962034</v>
+        <v>0.7745343920531087</v>
       </c>
       <c r="M8" t="n">
-        <v>0.01966583541848766</v>
+        <v>0.009357613120831939</v>
       </c>
     </row>
     <row r="9">
@@ -872,7 +872,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -882,29 +882,29 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G9" t="n">
         <v>5</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7499324435148262</v>
+        <v>0.768504717808238</v>
       </c>
       <c r="I9" t="n">
-        <v>0.02668125337544833</v>
+        <v>0.01619103553235011</v>
       </c>
       <c r="J9" t="n">
-        <v>0.7588571428571429</v>
+        <v>0.7542857142857142</v>
       </c>
       <c r="K9" t="n">
-        <v>0.01779704171702564</v>
+        <v>0.01399708424447527</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7542292479962034</v>
+        <v>0.7612597572519914</v>
       </c>
       <c r="M9" t="n">
-        <v>0.01966583541848766</v>
+        <v>0.01269023246414791</v>
       </c>
     </row>
     <row r="10">
@@ -925,7 +925,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -942,22 +942,22 @@
         <v>5</v>
       </c>
       <c r="H10" t="n">
-        <v>0.7979117605724549</v>
+        <v>0.7901920395695406</v>
       </c>
       <c r="I10" t="n">
-        <v>0.02630474341726022</v>
+        <v>0.03429817478840256</v>
       </c>
       <c r="J10" t="n">
-        <v>0.7929411764705883</v>
+        <v>0.7823529411764706</v>
       </c>
       <c r="K10" t="n">
-        <v>0.02054617552538</v>
+        <v>0.01315334104411645</v>
       </c>
       <c r="L10" t="n">
-        <v>0.7953442886268538</v>
+        <v>0.7858193909207959</v>
       </c>
       <c r="M10" t="n">
-        <v>0.02196473464022954</v>
+        <v>0.01504112554333517</v>
       </c>
     </row>
     <row r="11">
@@ -978,39 +978,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G11" t="n">
         <v>5</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7979117605724549</v>
+        <v>0.7796680784439497</v>
       </c>
       <c r="I11" t="n">
-        <v>0.02630474341726022</v>
+        <v>0.01490919711098299</v>
       </c>
       <c r="J11" t="n">
-        <v>0.7929411764705883</v>
+        <v>0.7858823529411765</v>
       </c>
       <c r="K11" t="n">
-        <v>0.02054617552538</v>
+        <v>0.01793876550820817</v>
       </c>
       <c r="L11" t="n">
-        <v>0.7953442886268538</v>
+        <v>0.7826344666569633</v>
       </c>
       <c r="M11" t="n">
-        <v>0.02196473464022954</v>
+        <v>0.01207496426143413</v>
       </c>
     </row>
     <row r="12">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1048,22 +1048,22 @@
         <v>5</v>
       </c>
       <c r="H12" t="n">
-        <v>0.7946384282584276</v>
+        <v>0.7934458801627304</v>
       </c>
       <c r="I12" t="n">
-        <v>0.02215577199420941</v>
+        <v>0.01532945167698434</v>
       </c>
       <c r="J12" t="n">
-        <v>0.7905882352941177</v>
+        <v>0.7858823529411765</v>
       </c>
       <c r="K12" t="n">
-        <v>0.01068582477916766</v>
+        <v>0.01068582477916762</v>
       </c>
       <c r="L12" t="n">
-        <v>0.7925445230105735</v>
+        <v>0.789627525125751</v>
       </c>
       <c r="M12" t="n">
-        <v>0.01535006605215245</v>
+        <v>0.01246544342141601</v>
       </c>
     </row>
     <row r="13">
@@ -1094,29 +1094,29 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G13" t="n">
         <v>5</v>
       </c>
       <c r="H13" t="n">
-        <v>0.7946384282584276</v>
+        <v>0.7824890253928366</v>
       </c>
       <c r="I13" t="n">
-        <v>0.02215577199420941</v>
+        <v>0.01433880487162856</v>
       </c>
       <c r="J13" t="n">
-        <v>0.7905882352941177</v>
+        <v>0.7870588235294118</v>
       </c>
       <c r="K13" t="n">
-        <v>0.01068582477916766</v>
+        <v>0.01464694070351622</v>
       </c>
       <c r="L13" t="n">
-        <v>0.7925445230105735</v>
+        <v>0.7847488058659879</v>
       </c>
       <c r="M13" t="n">
-        <v>0.01535006605215245</v>
+        <v>0.01387239862028402</v>
       </c>
     </row>
     <row r="14">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1151,25 +1151,25 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H14" t="n">
-        <v>0.8186567456362652</v>
+        <v>0.8147884327788443</v>
       </c>
       <c r="I14" t="n">
-        <v>0.007220599924965905</v>
+        <v>0.009756971543303797</v>
       </c>
       <c r="J14" t="n">
-        <v>0.8057142857142857</v>
+        <v>0.8045714285714286</v>
       </c>
       <c r="K14" t="n">
-        <v>0.008081220356417699</v>
+        <v>0.0130305762868473</v>
       </c>
       <c r="L14" t="n">
-        <v>0.812091021285785</v>
+        <v>0.8096412598311872</v>
       </c>
       <c r="M14" t="n">
-        <v>0.003552758547473675</v>
+        <v>0.01126940583748925</v>
       </c>
     </row>
     <row r="15">
@@ -1190,39 +1190,39 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G15" t="n">
         <v>5</v>
       </c>
       <c r="H15" t="n">
-        <v>0.8162890328726485</v>
+        <v>0.8101310710803645</v>
       </c>
       <c r="I15" t="n">
-        <v>0.008193480097753366</v>
+        <v>0.01798885220060057</v>
       </c>
       <c r="J15" t="n">
-        <v>0.8068571428571427</v>
+        <v>0.8045714285714286</v>
       </c>
       <c r="K15" t="n">
-        <v>0.007450517034517296</v>
+        <v>0.01869191683862417</v>
       </c>
       <c r="L15" t="n">
-        <v>0.8114961788519899</v>
+        <v>0.8073326312209611</v>
       </c>
       <c r="M15" t="n">
-        <v>0.003351978158894027</v>
+        <v>0.01810206853188335</v>
       </c>
     </row>
     <row r="16">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1260,22 +1260,22 @@
         <v>5</v>
       </c>
       <c r="H16" t="n">
-        <v>0.8157392026578073</v>
+        <v>0.823261689769366</v>
       </c>
       <c r="I16" t="n">
-        <v>0.01143414204462839</v>
+        <v>0.0175204085628956</v>
       </c>
       <c r="J16" t="n">
-        <v>0.7942857142857143</v>
+        <v>0.7965714285714285</v>
       </c>
       <c r="K16" t="n">
-        <v>0.0193780856660722</v>
+        <v>0.01251937274297525</v>
       </c>
       <c r="L16" t="n">
-        <v>0.8047992775629075</v>
+        <v>0.8095559633321203</v>
       </c>
       <c r="M16" t="n">
-        <v>0.01364890851437444</v>
+        <v>0.009390417384082165</v>
       </c>
     </row>
     <row r="17">
@@ -1306,29 +1306,29 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G17" t="n">
         <v>5</v>
       </c>
       <c r="H17" t="n">
-        <v>0.8157392026578073</v>
+        <v>0.8267651324193013</v>
       </c>
       <c r="I17" t="n">
-        <v>0.01143414204462839</v>
+        <v>0.01087867294839794</v>
       </c>
       <c r="J17" t="n">
-        <v>0.7942857142857143</v>
+        <v>0.801142857142857</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0193780856660722</v>
+        <v>0.01533303755999859</v>
       </c>
       <c r="L17" t="n">
-        <v>0.8047992775629075</v>
+        <v>0.8136648790207985</v>
       </c>
       <c r="M17" t="n">
-        <v>0.01364890851437444</v>
+        <v>0.009544293407475436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>